<commit_message>
Update test cases in Assignment 1 - Test cases.xlsx
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -632,22 +632,22 @@
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C3" s="16" t="inlineStr">
         <is>
-          <t>adha mokakda kare?</t>
+          <t>koheda yanawa da, api match eka balanna?</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>අද මොකක්ද කළේ?</t>
+          <t>කොහේද යනවා ද, අපි match එක බලන්න?</t>
         </is>
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>අද මොකක්ද කරේ?</t>
+          <t>කොහෙද යනවා ද, අපි match එක බලන්න?</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Rationale: Short question asking what was done today</t>
+          <t>Rationale: Longer question combining destination with a plan to watch a match</t>
         </is>
       </c>
     </row>
@@ -716,22 +716,22 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>phone dapanna.</t>
+          <t>phone dapanna, eka gena enna mama.</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>phone දාපන්නා.</t>
+          <t>phone දාපන්නා, ඒක ගෙන එන්නා මම.</t>
         </is>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>ෆෝන් දාපන්න.</t>
+          <t>ෆෝන් දාපන්න, ඒක ගැන එන්න මම.</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>Rationale: Short command to put the phone down</t>
+          <t>Rationale: Two chained commands — put down the phone and bring it here</t>
         </is>
       </c>
     </row>
@@ -800,22 +800,22 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>ayubovan machan!</t>
+          <t>ayubovan machan, kohomada oya unne?</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>ආයුබෝවන් මචන්!</t>
+          <t>ආයුබෝවන් මචන්, කොහොමද ඔය උන්නේ?</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>ආයුබෝවන් මචං!</t>
+          <t>ආයුබෝවන් මචං, කොහොමද ඔයා උන්නේ?</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>Rationale: Traditional greeting 'ayubovan' paired with informal 'machan'</t>
+          <t>Rationale: Traditional greeting 'ayubovan' followed by a casual how-are-you question</t>
         </is>
       </c>
     </row>
@@ -884,22 +884,22 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>poddak balanna.</t>
+          <t>poddak balanna, mama kiyannam eka.</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>පොඩ්ඩක් බලන්නා.</t>
+          <t>පොඩ්ඩක් බලන්නා, මම කියන්නම් ඒක.</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>පොඩ්ඩක් බලන්න.</t>
+          <t>පොඩ්ඩක් බලන්න, මම කියන්නම් ඒක.</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>Rationale: Polite two-word request to have a quick look</t>
+          <t>Rationale: Polite request to look followed by a promise to explain</t>
         </is>
       </c>
     </row>
@@ -968,22 +968,22 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>naha machan.</t>
+          <t>naha machan, mama danata enna bae.</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>නෑ මචන්.</t>
+          <t>නෑ මචන්, මම දැනට එන්නේ බෑ.</t>
         </is>
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>නැහැ මචං.</t>
+          <t>නැහැ මචං, මම දැනට එන්න බෑ.</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>Rationale: Negative response 'naha' (no) combined with slang 'machan'</t>
+          <t>Rationale: Negative response with explanation that coming right now is not possible</t>
         </is>
       </c>
     </row>
@@ -1052,27 +1052,27 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>loku loku epa.</t>
+          <t>loku loku karanawa epa, poddak kara.</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
+          <t>ලොකු ලොකු කරනවා එපා, පොඩ්ඩක් කරා.</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
           <t>ලොකු ලොකු එපා.</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>ලොකු ලොකු එපා.</t>
-        </is>
-      </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>UI Error</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="H13" s="16" t="inlineStr">
         <is>
-          <t>Rationale: 'loku loku' repeats 'loku' (big/major) for emphasis</t>
+          <t>Rationale: 'loku loku' emphatic repetition followed by a request to do it smaller</t>
         </is>
       </c>
     </row>
@@ -1136,27 +1136,27 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>ane! mokada?</t>
+          <t>ane! koheda una? api hora hora giya!</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>අනේ! මොකද?</t>
+          <t>අනේ! කොහේද උනා? අපි හොරා හොරා ගියා!</t>
         </is>
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>අනේ! මොකද?</t>
+          <t>අනේ! කොහෙද උනා? අපි හොරා හොරා ගියා!</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="H15" s="16" t="inlineStr">
         <is>
-          <t>Rationale: Input uses exclamation mark (!) and question mark (?)</t>
+          <t>Rationale: Input uses exclamation mark (!), question mark (?), and repeated exclamation</t>
         </is>
       </c>
     </row>
@@ -1220,22 +1220,22 @@
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>threi ne?</t>
+          <t>threi ne machan, mama kiwwe hari kiyala.</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>තේරෙයි නේ?</t>
+          <t>තේරෙයි නේ මචන්, මම කිව්වේ හරි කියලා.</t>
         </is>
       </c>
       <c r="E17" s="16" t="inlineStr">
         <is>
-          <t>ත්රී නේ?</t>
+          <t>ත්රීි නෑ මචං, මම කිව්වේ හරි කියලා.</t>
         </is>
       </c>
       <c r="F17" s="16" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="H17" s="16" t="inlineStr">
         <is>
-          <t>Rationale: 'threi' is a non-standard abbreviated spelling of 'therei' (understood)</t>
+          <t>Rationale: 'threi' is an abbreviated spelling of 'therei'; full sentence tests multi-word variant handling</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>UI Error</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
@@ -1388,22 +1388,22 @@
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>mama be right back.</t>
+          <t>mama be right back, poddak wait karanna.</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>මම be right back.</t>
+          <t>මම be right back, පොඩ්ඩක් wait කරන්නා.</t>
         </is>
       </c>
       <c r="E21" s="16" t="inlineStr">
         <is>
-          <t>මම බෑ right back.</t>
+          <t>මම බෑ right back, පොඩ්ඩක් wait කරන්න.</t>
         </is>
       </c>
       <c r="F21" s="16" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="H21" s="16" t="inlineStr">
         <is>
-          <t>Rationale: Multi-word English phrase 'be right back' embedded in Singlish</t>
+          <t>Rationale: English phrase 'be right back' combined with a Singlish request to wait</t>
         </is>
       </c>
     </row>
@@ -1472,27 +1472,27 @@
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>Bluetooth on kara.</t>
+          <t>Bluetooth on kara, speaker connect wenawada?</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>Bluetooth on කරා.</t>
+          <t>Bluetooth on කරා, speaker connect වෙනවාද?</t>
         </is>
       </c>
       <c r="E23" s="16" t="inlineStr">
         <is>
-          <t>Bluetooth on කරා.</t>
+          <t>Bluetooth on කරා, speaker connect වෙනවද?</t>
         </is>
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G23" s="16" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="H23" s="16" t="inlineStr">
         <is>
-          <t>Rationale: 'Bluetooth' is a digital term and 'on' is a technical command in Singlish</t>
+          <t>Rationale: Digital terms 'Bluetooth' and 'speaker' paired with a Singlish connectivity question</t>
         </is>
       </c>
     </row>
@@ -1556,22 +1556,22 @@
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>Telegram eke ewanna.</t>
+          <t>Telegram eke ewanna, group eke share kara.</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>Telegram එකේ එවන්නා.</t>
+          <t>Telegram එකේ එවන්නා, group එකේ share කරා.</t>
         </is>
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>Telegram එකේ එවන්න.</t>
+          <t>Telegram එකේ එවන්න, group එකේ share කරා.</t>
         </is>
       </c>
       <c r="F25" s="16" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="H25" s="16" t="inlineStr">
         <is>
-          <t>Rationale: 'Telegram' is an app name embedded in Singlish</t>
+          <t>Rationale: 'Telegram' app name with two chained Singlish actions — send and share</t>
         </is>
       </c>
     </row>
@@ -1640,22 +1640,22 @@
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>ASAP ewanna.</t>
+          <t>ASAP ewanna, project deadline innawa.</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>ASAP එවන්නා.</t>
+          <t>ASAP එවන්නා, project deadline ඉන්නවා.</t>
         </is>
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>ASAP එවන්න.</t>
+          <t>ASAP එවන්න, project deadline ඉන්නවා.</t>
         </is>
       </c>
       <c r="F27" s="16" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H27" s="16" t="inlineStr">
         <is>
-          <t>Rationale: 'ASAP' (As Soon As Possible) is an English acronym in Singlish</t>
+          <t>Rationale: 'ASAP' acronym combined with a project deadline context in Singlish</t>
         </is>
       </c>
     </row>
@@ -2060,22 +2060,22 @@
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>USD 10 denna.</t>
+          <t>USD 10 denna mama, rate eka check kara.</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>USD 10 දෙන්නා.</t>
+          <t>USD 10 දෙන්නා මම, rate එක check කරා.</t>
         </is>
       </c>
       <c r="E37" s="16" t="inlineStr">
         <is>
-          <t>USD 10 දෙන්න.</t>
+          <t>USD 10 දෙන්න මම, rate එක check කරා.</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="H37" s="16" t="inlineStr">
         <is>
-          <t>Rationale: 'USD' is a foreign currency code embedded in Singlish</t>
+          <t>Rationale: Foreign currency 'USD' combined with a Singlish instruction to check the rate</t>
         </is>
       </c>
     </row>
@@ -2144,22 +2144,22 @@
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>9:00AM meeting eka.</t>
+          <t>9:00AM meeting eka thiyanawa machan.</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>9:00AM meeting එකා.</t>
+          <t>9:00AM meeting එකා තියනවා මචන්.</t>
         </is>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
-          <t>9:00AM meeting එක.</t>
+          <t>9:00AM meeting එක තියෙනවා මචන්.</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="H39" s="16" t="inlineStr">
         <is>
-          <t>Rationale: '9:00AM' is a time format combined with Singlish text</t>
+          <t>Rationale: '9:00AM' time format combined with Singlish informal address 'machan'</t>
         </is>
       </c>
     </row>
@@ -2396,22 +2396,22 @@
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>sirawata set.</t>
+          <t>sirawata set bro, oyage dance eka patta.</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>සිරාවට සෙට්.</t>
+          <t>සිරාවට සෙට් bro, ඔයාගේ dance එක පට්ට.</t>
         </is>
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>සිරාවට set.</t>
+          <t>සිරාවට set bro, ඔයාගෙ dance එක පට්ට.</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="H45" s="16" t="inlineStr">
         <is>
-          <t>Rationale: 'sirawata' (truly/really) and 'set' (cool/crew) are casual Singlish slang terms</t>
+          <t>Rationale: 'sirawata set' and 'patta' are casual slang terms praising a dance performance</t>
         </is>
       </c>
     </row>

</xml_diff>